<commit_message>
Ver 2.0 Added Overtime Filing
</commit_message>
<xml_diff>
--- a/Yondu Timesheet_Novemberr 1-15 2021_Monica Cho.xlsx
+++ b/Yondu Timesheet_Novemberr 1-15 2021_Monica Cho.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Snow\projects_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1778569-F38F-4095-ADCB-282984CDF8A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF7D41D-34AF-441C-B95B-62573CDF1057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="51">
   <si>
     <t>DAILY TIMESHEET</t>
   </si>
@@ -171,7 +171,19 @@
     <t>9/17/2021</t>
   </si>
   <si>
-    <t>On Leave</t>
+    <t>05/16/2022 Mon</t>
+  </si>
+  <si>
+    <t>05/17/2022 Tue</t>
+  </si>
+  <si>
+    <t>05/18/2022 Wed</t>
+  </si>
+  <si>
+    <t>05/19/2022 Thu</t>
+  </si>
+  <si>
+    <t>Weekend Support</t>
   </si>
 </sst>
 </file>
@@ -543,40 +555,40 @@
     <xf numFmtId="18" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="15" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,27 +818,27 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
-      <c r="S1" s="58"/>
-      <c r="T1" s="59"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="44"/>
       <c r="U1" s="2"/>
       <c r="V1" s="2"/>
       <c r="W1" s="2"/>
@@ -867,26 +879,26 @@
       <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="54" t="s">
+      <c r="C3" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="47"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="45" t="s">
+      <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="50"/>
-      <c r="L3" s="54" t="s">
+      <c r="K3" s="49"/>
+      <c r="L3" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="43"/>
-      <c r="N3" s="43"/>
-      <c r="O3" s="43"/>
-      <c r="P3" s="44"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
+      <c r="P3" s="47"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
@@ -903,26 +915,26 @@
       <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="54" t="s">
+      <c r="C4" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="44"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="47"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="45" t="s">
+      <c r="J4" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="50"/>
-      <c r="L4" s="54" t="s">
+      <c r="K4" s="49"/>
+      <c r="L4" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="43"/>
-      <c r="N4" s="43"/>
-      <c r="O4" s="43"/>
-      <c r="P4" s="44"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="47"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
@@ -939,26 +951,26 @@
       <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="54" t="s">
+      <c r="C5" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
       <c r="I5" s="4"/>
-      <c r="J5" s="45" t="s">
+      <c r="J5" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="50"/>
-      <c r="L5" s="54" t="s">
+      <c r="K5" s="49"/>
+      <c r="L5" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="43"/>
-      <c r="N5" s="43"/>
-      <c r="O5" s="43"/>
-      <c r="P5" s="44"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="47"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
@@ -975,17 +987,17 @@
       <c r="B6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="47"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="50"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="49"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
@@ -1032,46 +1044,46 @@
     </row>
     <row r="8" spans="1:26" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="55" t="s">
+      <c r="C8" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="48"/>
-      <c r="M8" s="53" t="s">
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="46"/>
+      <c r="J8" s="46"/>
+      <c r="K8" s="46"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="N8" s="53" t="s">
+      <c r="N8" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="O8" s="53" t="s">
+      <c r="O8" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="P8" s="53" t="s">
+      <c r="P8" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="Q8" s="53" t="s">
+      <c r="Q8" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="R8" s="53" t="s">
+      <c r="R8" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="S8" s="53" t="s">
+      <c r="S8" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="T8" s="53" t="s">
+      <c r="T8" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="U8" s="53" t="s">
+      <c r="U8" s="50" t="s">
         <v>24</v>
       </c>
       <c r="V8" s="4"/>
@@ -1082,7 +1094,7 @@
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
-      <c r="B9" s="48"/>
+      <c r="B9" s="51"/>
       <c r="C9" s="8" t="s">
         <v>25</v>
       </c>
@@ -1113,15 +1125,15 @@
       <c r="L9" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="M9" s="48"/>
-      <c r="N9" s="47"/>
-      <c r="O9" s="47"/>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="48"/>
-      <c r="R9" s="48"/>
-      <c r="S9" s="48"/>
-      <c r="T9" s="48"/>
-      <c r="U9" s="48"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="53"/>
+      <c r="O9" s="53"/>
+      <c r="P9" s="51"/>
+      <c r="Q9" s="51"/>
+      <c r="R9" s="51"/>
+      <c r="S9" s="51"/>
+      <c r="T9" s="51"/>
+      <c r="U9" s="51"/>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
@@ -1130,8 +1142,8 @@
     </row>
     <row r="10" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="7"/>
-      <c r="B10" s="9">
-        <v>44697</v>
+      <c r="B10" s="9" t="s">
+        <v>46</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>31</v>
@@ -1139,13 +1151,13 @@
       <c r="D10" s="11">
         <v>8</v>
       </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
       <c r="L10" s="11"/>
       <c r="M10" s="11">
         <v>8</v>
@@ -1172,8 +1184,8 @@
     </row>
     <row r="11" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="7"/>
-      <c r="B11" s="9">
-        <v>44698</v>
+      <c r="B11" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>31</v>
@@ -1181,13 +1193,13 @@
       <c r="D11" s="11">
         <v>8</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
       <c r="L11" s="11"/>
       <c r="M11" s="11">
         <v>8</v>
@@ -1214,8 +1226,8 @@
     </row>
     <row r="12" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="34"/>
-      <c r="B12" s="9">
-        <v>44699</v>
+      <c r="B12" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>31</v>
@@ -1256,9 +1268,15 @@
     </row>
     <row r="13" spans="1:26" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="34"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="11"/>
+      <c r="B13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="11">
+        <v>6</v>
+      </c>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
@@ -1267,15 +1285,25 @@
       <c r="J13" s="16"/>
       <c r="K13" s="16"/>
       <c r="L13" s="16"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="39"/>
-      <c r="O13" s="39"/>
-      <c r="P13" s="11"/>
+      <c r="M13" s="11">
+        <v>6</v>
+      </c>
+      <c r="N13" s="40">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="O13" s="40">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="P13" s="11">
+        <v>6</v>
+      </c>
       <c r="Q13" s="19"/>
       <c r="R13" s="36"/>
       <c r="S13" s="32"/>
       <c r="T13" s="32"/>
-      <c r="U13" s="16"/>
+      <c r="U13" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="V13" s="18"/>
       <c r="W13" s="18"/>
       <c r="X13" s="18"/>
@@ -1415,9 +1443,7 @@
       <c r="R18" s="33"/>
       <c r="S18" s="33"/>
       <c r="T18" s="15"/>
-      <c r="U18" s="15" t="s">
-        <v>46</v>
-      </c>
+      <c r="U18" s="15"/>
       <c r="V18" s="22"/>
       <c r="W18" s="22"/>
       <c r="X18" s="22"/>
@@ -1600,7 +1626,7 @@
       <c r="C25" s="20"/>
       <c r="D25" s="8">
         <f>SUM(D10:D20)</f>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E25" s="20"/>
       <c r="F25" s="8">
@@ -1624,13 +1650,13 @@
       </c>
       <c r="M25" s="8">
         <f>SUM(M10:M20)</f>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="N25" s="20"/>
       <c r="O25" s="20"/>
       <c r="P25" s="8">
         <f>SUM(P10:P20)</f>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="Q25" s="8">
         <f>SUM(Q10:Q20)</f>
@@ -1800,30 +1826,30 @@
       <c r="B31" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C31" s="49" t="s">
+      <c r="C31" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="44"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="47"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="45" t="s">
+      <c r="J31" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="K31" s="50"/>
-      <c r="L31" s="52" t="s">
+      <c r="K31" s="49"/>
+      <c r="L31" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="M31" s="43"/>
-      <c r="N31" s="43"/>
-      <c r="O31" s="43"/>
-      <c r="P31" s="43"/>
-      <c r="Q31" s="43"/>
-      <c r="R31" s="43"/>
-      <c r="S31" s="43"/>
-      <c r="T31" s="44"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="46"/>
+      <c r="Q31" s="46"/>
+      <c r="R31" s="46"/>
+      <c r="S31" s="46"/>
+      <c r="T31" s="47"/>
       <c r="U31" s="4"/>
       <c r="V31" s="4"/>
       <c r="W31" s="4"/>
@@ -1861,29 +1887,29 @@
     </row>
     <row r="33" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
-      <c r="B33" s="51" t="s">
+      <c r="B33" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="C33" s="46"/>
-      <c r="D33" s="46"/>
-      <c r="E33" s="46"/>
-      <c r="F33" s="46"/>
-      <c r="G33" s="46"/>
-      <c r="H33" s="46"/>
-      <c r="I33" s="47"/>
-      <c r="J33" s="51" t="s">
+      <c r="C33" s="57"/>
+      <c r="D33" s="57"/>
+      <c r="E33" s="57"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="57"/>
+      <c r="H33" s="57"/>
+      <c r="I33" s="53"/>
+      <c r="J33" s="56" t="s">
         <v>36</v>
       </c>
-      <c r="K33" s="46"/>
-      <c r="L33" s="46"/>
-      <c r="M33" s="46"/>
-      <c r="N33" s="46"/>
-      <c r="O33" s="46"/>
-      <c r="P33" s="46"/>
-      <c r="Q33" s="46"/>
-      <c r="R33" s="46"/>
-      <c r="S33" s="46"/>
-      <c r="T33" s="47"/>
+      <c r="K33" s="57"/>
+      <c r="L33" s="57"/>
+      <c r="M33" s="57"/>
+      <c r="N33" s="57"/>
+      <c r="O33" s="57"/>
+      <c r="P33" s="57"/>
+      <c r="Q33" s="57"/>
+      <c r="R33" s="57"/>
+      <c r="S33" s="57"/>
+      <c r="T33" s="53"/>
       <c r="U33" s="4"/>
       <c r="V33" s="4"/>
       <c r="W33" s="4"/>
@@ -1929,21 +1955,21 @@
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="21"/>
-      <c r="J35" s="45" t="s">
+      <c r="J35" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="K35" s="46"/>
-      <c r="L35" s="47"/>
+      <c r="K35" s="57"/>
+      <c r="L35" s="53"/>
       <c r="M35" s="4"/>
-      <c r="N35" s="42"/>
-      <c r="O35" s="43"/>
-      <c r="P35" s="44"/>
+      <c r="N35" s="58"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="47"/>
       <c r="Q35" s="4"/>
       <c r="R35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="S35" s="42"/>
-      <c r="T35" s="48"/>
+      <c r="S35" s="58"/>
+      <c r="T35" s="51"/>
       <c r="U35" s="4"/>
       <c r="V35" s="4"/>
       <c r="W35" s="4"/>
@@ -1953,33 +1979,33 @@
     </row>
     <row r="36" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="7"/>
-      <c r="B36" s="45" t="s">
+      <c r="B36" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="47"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="44"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="58"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="47"/>
       <c r="G36" s="4" t="s">
         <v>38</v>
       </c>
       <c r="H36" s="6"/>
       <c r="I36" s="12"/>
-      <c r="J36" s="45" t="s">
+      <c r="J36" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="K36" s="46"/>
-      <c r="L36" s="47"/>
+      <c r="K36" s="57"/>
+      <c r="L36" s="53"/>
       <c r="M36" s="4"/>
-      <c r="N36" s="42"/>
-      <c r="O36" s="43"/>
-      <c r="P36" s="44"/>
+      <c r="N36" s="58"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="47"/>
       <c r="Q36" s="4"/>
       <c r="R36" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="S36" s="42"/>
-      <c r="T36" s="48"/>
+      <c r="S36" s="58"/>
+      <c r="T36" s="51"/>
       <c r="U36" s="4"/>
       <c r="V36" s="4"/>
       <c r="W36" s="4"/>
@@ -1997,21 +2023,21 @@
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="21"/>
-      <c r="J37" s="45" t="s">
+      <c r="J37" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="K37" s="46"/>
-      <c r="L37" s="47"/>
+      <c r="K37" s="57"/>
+      <c r="L37" s="53"/>
       <c r="M37" s="4"/>
-      <c r="N37" s="42"/>
-      <c r="O37" s="43"/>
-      <c r="P37" s="44"/>
+      <c r="N37" s="58"/>
+      <c r="O37" s="46"/>
+      <c r="P37" s="47"/>
       <c r="Q37" s="4"/>
       <c r="R37" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="S37" s="42"/>
-      <c r="T37" s="48"/>
+      <c r="S37" s="58"/>
+      <c r="T37" s="51"/>
       <c r="U37" s="4"/>
       <c r="V37" s="4"/>
       <c r="W37" s="4"/>
@@ -2021,33 +2047,33 @@
     </row>
     <row r="38" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="7"/>
-      <c r="B38" s="45" t="s">
+      <c r="B38" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="C38" s="47"/>
-      <c r="D38" s="42"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="44"/>
+      <c r="C38" s="53"/>
+      <c r="D38" s="58"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="47"/>
       <c r="G38" s="4" t="s">
         <v>38</v>
       </c>
       <c r="H38" s="6"/>
       <c r="I38" s="12"/>
-      <c r="J38" s="45" t="s">
+      <c r="J38" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="K38" s="46"/>
-      <c r="L38" s="47"/>
+      <c r="K38" s="57"/>
+      <c r="L38" s="53"/>
       <c r="M38" s="4"/>
-      <c r="N38" s="42"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="44"/>
+      <c r="N38" s="58"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="47"/>
       <c r="Q38" s="4"/>
       <c r="R38" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="S38" s="42"/>
-      <c r="T38" s="48"/>
+      <c r="S38" s="58"/>
+      <c r="T38" s="51"/>
       <c r="U38" s="4"/>
       <c r="V38" s="4"/>
       <c r="W38" s="4"/>
@@ -2065,21 +2091,21 @@
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="21"/>
-      <c r="J39" s="45" t="s">
+      <c r="J39" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="K39" s="46"/>
-      <c r="L39" s="47"/>
+      <c r="K39" s="57"/>
+      <c r="L39" s="53"/>
       <c r="M39" s="4"/>
-      <c r="N39" s="42"/>
-      <c r="O39" s="43"/>
-      <c r="P39" s="44"/>
+      <c r="N39" s="58"/>
+      <c r="O39" s="46"/>
+      <c r="P39" s="47"/>
       <c r="Q39" s="4"/>
       <c r="R39" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="S39" s="42"/>
-      <c r="T39" s="48"/>
+      <c r="S39" s="58"/>
+      <c r="T39" s="51"/>
       <c r="U39" s="4"/>
       <c r="V39" s="4"/>
       <c r="W39" s="4"/>
@@ -28745,29 +28771,16 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="B1:T1"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L3:P3"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="L4:P4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L5:P5"/>
-    <mergeCell ref="C5:H5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:L8"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="N39:P39"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="J37:L37"/>
+    <mergeCell ref="N37:P37"/>
+    <mergeCell ref="S37:T37"/>
+    <mergeCell ref="J38:L38"/>
+    <mergeCell ref="S38:T38"/>
+    <mergeCell ref="J39:L39"/>
+    <mergeCell ref="S39:T39"/>
+    <mergeCell ref="S36:T36"/>
     <mergeCell ref="C31:H31"/>
     <mergeCell ref="J31:K31"/>
     <mergeCell ref="B33:I33"/>
@@ -28782,16 +28795,29 @@
     <mergeCell ref="J35:L35"/>
     <mergeCell ref="N35:P35"/>
     <mergeCell ref="S35:T35"/>
-    <mergeCell ref="N39:P39"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="J37:L37"/>
-    <mergeCell ref="N37:P37"/>
-    <mergeCell ref="S37:T37"/>
-    <mergeCell ref="J38:L38"/>
-    <mergeCell ref="S38:T38"/>
-    <mergeCell ref="J39:L39"/>
-    <mergeCell ref="S39:T39"/>
-    <mergeCell ref="S36:T36"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="S8:S9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="L5:P5"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:L8"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="B1:T1"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="L3:P3"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="L4:P4"/>
+    <mergeCell ref="J4:K4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>